<commit_message>
Add Durian, Fish Sauce Mike, Matcha, Chrysanthemum, Squid, and Chocolate to affiliate products
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1323,6 +1323,186 @@
       <c r="F20" s="5" t="inlineStr">
         <is>
           <t>ลด 20% วันนี้เท่านั้น</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>❤️ส่งด่วน1วัน รีวิวเยอะสุด 🙏เกรดพรีเมี่ยม ทุเรียนหมอนทองจันทบุรี แกะเนื้อล้วน พร้อมทาน 🚚ส่งรถเย็น</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8V637eNSrM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>ทุเรียนหมอนทองจันทบุรี แกะเนื้อล้วน พร้อมทาน ส่งเย็นสดๆ</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>[✅โค้ดส่งฟรี+🎫โค้ดคุุ้ม] น้ำปลาร้าปรุงสุก ตราไมค์ 6 ขวด ขนาด 350 ml. (แซ่บไมค์) น้ำปลาร้า ปรุงสุก สูตรแซ่บทุกเมนู</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/809mXCj4Pw</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>น้ำปลาร้าปรุงสุกแซ่บไมค์ 6 ขวด นัวทุกครก แซ่บทุกเมนู</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>6</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ชาเขียว 100% เพียวมัทฉะ ชาเขียว พรีเมี่ยม matcha powder from japan 0 สารเติมแต่ง 1 กระป๋อง 300g</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8V6389O8pb</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>ผงมัทฉะแท้ 100% พรีเมี่ยม นำเข้าจากญี่ปุ่น เข้มข้นกลมกล่อม</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>7</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>เก๊กฮวยผงสำเร็จรูป HighlandHerb ขนาด 600 กรัม</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/6VKykVDy1E</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>เก๊กฮวยผงสำเร็จรูป HighlandHerb ชงง่าย หอมสดชื่น ดับกระหาย</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>8</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ปลาหมึกแห้ง ปลาหมึกแพไข่ ไซส์กลาง ไม่เค็มมาก ตากสดใหม่ รับประกันความอร่อย</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/50WAxlk5Hu</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>ปลาหมึกแห้งแพไข่ ไซส์กลาง สดใหม่ ไม่เค็มมาก อร่อยฟิน</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>9</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>🍫ขายร้อน🍫ช็อกโกแลต ดาร์กช็อกโกแลตฟิตเนส ไขมันต่ำ ขมสุด ไม่มีน้ำตาล ลดน้ำหนัก ดาร์กช็อกโกแลตแท้ 100%</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8pitWqXhxW</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>ดาร์กช็อกโกแลตแท้ 100% คีโตทานได้ ไม่มีน้ำตาล คุมน้ำหนัก</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ShopeeFood 50% discount promotion (Chester's, Potato Corner, etc.)
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -934,6 +934,40 @@
           <t>ลองเข้ามาดู ขาหมูชานเมือง ข้าวมันไก่ อาหารตามสั่ง ก๋วยเตี๋ยว ที่ Shopee! https://spf.shopee.co.th/AAE8Lxgj6W</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>📍ปักหมุด แบรนด์ดังลดแรง 50% แถมใช้โค้ดลดเพิ่มได้อีก 60% สั่งเลยที่ ShopeeFood 👉 https://spf.shopee.co.th/40ddmXtVay
+.
+อร่อยฟินทั้งวีคกับเมนูฮิตจาก Chester's, Potato Corner, Swensen's, Sizzler, D'Oro
+.
+อย่าลืมคุ้ม 2 ต่อ
+✅สั่งเมนูลดสูงสุด 50%
+✅ใช้โค้ดลดเพิ่ม 60%
+.
+📆 ตั้งแต่วันที่ 25 พ.ค. 69 - 31 พ.ค. 69  เท่านั้น
+*อ่านเงื่อนไขเพิ่มเติมในหน้ากิจกรรม</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://spf.shopee.co.th/40ddmXtVay</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://scontent.fbkk5-8.fna.fbcdn.net/v/t39.30808-6/705682162_1435181848647581_7031149084495471946_n.jpg?_nc_cat=106&amp;ccb=1-7&amp;_nc_sid=127cfc&amp;_nc_ohc=dx6ZSuAsrVoQ7kNvwGjkgf3&amp;_nc_oc=AdoTnyNM99BKbNf9JX4bF76_THLmEwWIPQk2c5p5_j-WWwdsvDiOVuFGkExvBAPGHn02xO2RD8wX3dXjWIJ4djYI&amp;_nc_zt=23&amp;_nc_ht=scontent.fbkk5-8.fna&amp;_nc_gid=YnlhUQJ7r9ERLWtRnFD8Tw&amp;_nc_ss=7b2a8&amp;oh=00_Af5VXjSJ2ETwfBEJv1Fv8nHb_BzZyUGnTkmMLks3wVZrdA&amp;oe=6A1A3C0A</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="B8" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update affiliate products - add Durian Monthong (new URL)
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1537,6 +1537,36 @@
       <c r="F26" t="inlineStr">
         <is>
           <t>ดาร์กช็อกโกแลตแท้ 100% คีโตทานได้ ไม่มีน้ำตาล คุมน้ำหนัก</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>10</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ส่งด่วน1วัน เกรดพรีเมี่ยม ทุเรียนหมอนทองจันทบุรี แกะเนื้อล้วน พร้อมทาน ส่งรถเย็น</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7VDZJLoJYK</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>ทุเรียนหมอนทองจันทบุรี แกะเนื้อล้วน พร้อมทาน หวานมันกรอบนอกนุ่มใน ส่งรถเย็นถึงบ้าน</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update affiliate products - add KFC, Coke Brand Week, and Fuku Matcha promotions
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -1000,6 +1000,39 @@
           <t>ลองเข้ามาดู ข้าวหมูทอดอร่อยมาก ที่ Shopee! https://spf.shopee.co.th/BQmRZCjn6</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>โปรนี้มันคุ้มเกินต้าน! ไก่ทอดเน้นๆ วิงซ์แซ่บซี๊ดๆ 👉🏻 https://spf.shopee.co.th/4qCo97uUd7
+KFC จัดโปรท้าหน้าฝนสุดคุ้ม เฉพาะลูกค้า ShopeeFood เท่านั้น
+🍗 จัดใหญ่ในราคา 199.- (จากปกติ 275.-)
+💰 พิเศษ! ใช้ COINS ลดเพิ่ม เหลือเพียง 100.-
+กดสั่งเลยที่ ShopeeFood
+*ราคาหลังใช้โค้ดส่วนลดและ coins โค้ดส่วนลดมีจำนวนจำกัด อ่านเงื่อนไขเพิ่มเติมในหน้าร้านค้า
+#ShopeeFoodTH
+#ShopeeFoodเลือกถูกทุกมื้อ
+#เปิดShopeeกดซ้ายบนสั่งShopeeFood</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://spf.shopee.co.th/4qCo97uUd7</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://scontent.fbkk5-6.fna.fbcdn.net/v/t39.30808-6/708223404_1437030405129392_4428869259083351006_n.jpg?_nc_cat=102&amp;ccb=1-7&amp;_nc_sid=127cfc&amp;_nc_ohc=sb4nOoC7XfEQ7kNvwGctKR8&amp;_nc_oc=Adrg29wfG9Kr-WhvhPRmLmw0Rws7VWvRl3QTMdq6vr6-eEmyFJ9XeWT0dVnW87utfW-zxuHFWbCYapevqb7mDOeT&amp;_nc_zt=23&amp;_nc_ht=scontent.fbkk5-6.fna&amp;_nc_gid=0NAArV2aaNR4-rI8ck88OA&amp;_nc_ss=7b2a8&amp;oh=00_Af5ts38spEpZ084OvUXh_G3eFerKMI_h4xGkNBvkVjQ0vA&amp;oe=6A1D030F</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="B9" s="6" t="inlineStr">
@@ -1032,6 +1065,36 @@
           <t>ลองเข้ามาดู Chester's ที่ Shopee! https://spf.shopee.co.th/9pbHxIUZ3g</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>💥 Coke x Brand Week อร่อยซ่ากับโค้ก แจกโค้ดลด 35.- ขั้นต่ำ 100.- ใช้โค้ด 'COKEBW54' รีบกดสั่งเลย 👉 https://s.shopee.co.th/2BC2yK1jwA
+.
+💥เฉพาะเมนูอร่อยซ่ากับโค้กจาก Chester's และ Sizzler
+.
+📆 ตั้งแต่วันที่ 25 พ.ค. 69 - 31 พ.ค. 69  เท่านั้น
+*อ่านเงื่อนไขเพิ่มเติมในหน้ากิจกรรม</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/2BC2yK1jwA</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://scontent.fbkk5-8.fna.fbcdn.net/v/t39.30808-6/706029253_1436136731885426_8787299363320150021_n.jpg?_nc_cat=106&amp;ccb=1-7&amp;_nc_sid=127cfc&amp;_nc_ohc=IS-SwDfJws8Q7kNvwE2BQeY&amp;_nc_oc=AdpXRsj7ZHTfhmHxdLJ20fFAF4rxevufcdOuaadzXKN6SMP089sgPCYJduNbbgsv37L5lKDKS-Qjw53h2d4wbevj&amp;_nc_zt=23&amp;_nc_ht=scontent.fbkk5-8.fna&amp;_nc_gid=HGF7KiF-72yMPCDoUwtCEw&amp;_nc_ss=7b2a8&amp;oh=00_Af5Y6aTOtoGIMh0H0jDXFAYl0kZhTBL5JUSRiNp2S6m96g&amp;oe=6A1CF9D6</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="B10" s="6" t="inlineStr">
@@ -1062,6 +1125,37 @@
       <c r="G10" t="inlineStr">
         <is>
           <t>ลองเข้ามาดู McDonald's ที่ Shopee! https://spf.shopee.co.th/3B4O11yxCV</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>🧡 Fuku Matcha 1 แถม 1 !!  แค่ 3 วันเท่านั้น! 😋 เฉพาะที่ ShopeeFood สั่งเลย 👉🏻 https://spf.shopee.co.th/6VL28LO6tD
+.
+✨ ต่อที่ 1: Double Black Milk Tea 1 แถม 1 ลดเหลือ 85.- (ตกแก้วละ 43.-)  จากปกติ 170.- 
+✨ ต่อที่ 2: ใช้ Coins ลดเพิ่มได้อีกสูงสุด 50% ของราคาอาหาร (สูงสุด 500 Coins ต่อวัน)
+. 
+📆 เฉพาะวันที่ 26 พ.ค. 69 - 28 พ.ค. 69 เท่านั้น
+*โค้ดส่วนลดมีจำนวนจำกัด อ่านเงื่อนไขเพิ่มเติมในหน้าร้านค้า, เฉพาะสาขาที่ร่วมรายการ</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://spf.shopee.co.th/6VL28LO6tD</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://scontent.fbkk5-7.fna.fbcdn.net/v/t39.30808-6/706464519_1435824978583268_8348776395536801292_n.jpg?_nc_cat=107&amp;ccb=1-7&amp;_nc_sid=127cfc&amp;_nc_ohc=Vb3ejVxYMJwQ7kNvwFP6Njh&amp;_nc_oc=AdpMTECmv7DCQJPwbiNz1tYIPpn018dpHzrkFg29IlaJ4CP79nDMw8ngnI7n1v2dis4ZQ2GYzvVtFFsrL-uTDbRF&amp;_nc_zt=23&amp;_nc_ht=scontent.fbkk5-7.fna&amp;_nc_gid=byYgzK1ChdSmBMbRWxdg7A&amp;_nc_ss=7b2a8&amp;oh=00_Af6pxydblvBJ1mr4MEtaNw-D0EyfuYTJK4lhNsVbIrc9VA&amp;oe=6A1CD07C</t>
         </is>
       </c>
     </row>

</xml_diff>